<commit_message>
Moved salary processing before standard processing
</commit_message>
<xml_diff>
--- a/instruction_data/templates/output_template.xlsx
+++ b/instruction_data/templates/output_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyle/projects/onesky_financial_agent/instruction_data/raw_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyle/projects/onesky_financial_agent/instruction_data/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7599B972-A8EB-874A-BC77-48B0A21C461F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{236E2284-B87B-B645-858E-AF849AAAB3B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1480" windowWidth="27240" windowHeight="15020" xr2:uid="{B9A37C1C-BF88-8C47-B40E-B31392CA78A1}"/>
+    <workbookView xWindow="12800" yWindow="1300" windowWidth="27240" windowHeight="15020" xr2:uid="{B9A37C1C-BF88-8C47-B40E-B31392CA78A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -66,7 +66,7 @@
     <definedName name="YTDCashBalance">#REF!</definedName>
     <definedName name="YTDMonthOfCash">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="66">
   <si>
     <t>Ending Balance</t>
   </si>
@@ -251,9 +251,6 @@
     <t>I.B</t>
   </si>
   <si>
-    <t>PED</t>
-  </si>
-  <si>
     <t>Interest</t>
   </si>
   <si>
@@ -285,6 +282,9 @@
   </si>
   <si>
     <t>Manual input</t>
+  </si>
+  <si>
+    <t>Cash settlement</t>
   </si>
 </sst>
 </file>
@@ -892,34 +892,34 @@
   <sheetData>
     <row r="1" spans="1:5" ht="29" x14ac:dyDescent="0.2">
       <c r="D1" s="21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D2" s="20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="22"/>
       <c r="B3" s="22"/>
       <c r="C3" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B4" s="8"/>
       <c r="C4" s="14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -927,10 +927,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -938,10 +938,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -949,21 +949,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="12">
         <v>4</v>
       </c>
-      <c r="B8" s="17" t="s">
-        <v>54</v>
-      </c>
+      <c r="B8" s="17"/>
       <c r="C8" s="16" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -1278,7 +1276,7 @@
     <row r="40" spans="1:4" ht="16" thickTop="1" x14ac:dyDescent="0.2"/>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C41" s="23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D41" s="23"/>
     </row>

</xml_diff>

<commit_message>
Update dec files and edit manual logic
</commit_message>
<xml_diff>
--- a/instruction_data/templates/output_template.xlsx
+++ b/instruction_data/templates/output_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyle/projects/onesky_financial_agent/instruction_data/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2783EADD-5FA7-324A-8F63-0C807542AE9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2523AE63-4A45-414F-B9DD-B8562BF335AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8600" yWindow="1180" windowWidth="27240" windowHeight="15020" xr2:uid="{B9A37C1C-BF88-8C47-B40E-B31392CA78A1}"/>
+    <workbookView xWindow="1560" yWindow="1180" windowWidth="27240" windowHeight="15020" xr2:uid="{B9A37C1C-BF88-8C47-B40E-B31392CA78A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="68">
   <si>
     <t>Ending Balance</t>
   </si>
@@ -285,6 +285,12 @@
   </si>
   <si>
     <t>Province Manual</t>
+  </si>
+  <si>
+    <t>IV</t>
+  </si>
+  <si>
+    <t>PAYABLE</t>
   </si>
 </sst>
 </file>
@@ -481,7 +487,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -548,6 +554,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="2" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1268,15 +1280,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="1" t="s">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="B39" s="25"/>
+      <c r="C39" s="25" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="16" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:4" ht="16" thickTop="1" x14ac:dyDescent="0.2">
       <c r="C41" s="23" t="s">
         <v>63</v>
       </c>

</xml_diff>

<commit_message>
Add support for Bank 34 transactions and enhance exchange rate handling
</commit_message>
<xml_diff>
--- a/instruction_data/templates/output_template.xlsx
+++ b/instruction_data/templates/output_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyle/projects/onesky_financial_agent/instruction_data/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2523AE63-4A45-414F-B9DD-B8562BF335AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B3EF303-9ADC-D04B-8243-7E8689EEFE9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1560" yWindow="1180" windowWidth="27240" windowHeight="15020" xr2:uid="{B9A37C1C-BF88-8C47-B40E-B31392CA78A1}"/>
   </bookViews>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="69">
   <si>
     <t>Ending Balance</t>
   </si>
@@ -291,6 +291,9 @@
   </si>
   <si>
     <t>PAYABLE</t>
+  </si>
+  <si>
+    <t>Vietcombank - ELC</t>
   </si>
 </sst>
 </file>
@@ -896,36 +899,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0458A968-68B9-CD41-AD6C-57431328A921}">
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="24.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="29" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="29" x14ac:dyDescent="0.2">
       <c r="D1" s="21" t="s">
         <v>61</v>
       </c>
       <c r="E1" s="21" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F1" s="21" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="D2" s="20" t="s">
         <v>59</v>
       </c>
       <c r="E2" s="20" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F2" s="20" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="22"/>
       <c r="B3" s="22"/>
       <c r="C3" s="7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
         <v>58</v>
       </c>
@@ -934,7 +943,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="12">
         <v>1</v>
       </c>
@@ -945,7 +954,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="12">
         <v>2</v>
       </c>
@@ -956,7 +965,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="12">
         <v>3</v>
       </c>
@@ -967,7 +976,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="12">
         <v>4</v>
       </c>
@@ -976,7 +985,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="19" t="s">
         <v>52</v>
       </c>
@@ -985,7 +994,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="12">
         <v>1</v>
       </c>
@@ -996,12 +1005,12 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="10"/>
       <c r="B11" s="10"/>
       <c r="C11" s="15"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="8" t="s">
         <v>48</v>
       </c>
@@ -1010,7 +1019,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="12">
         <v>1</v>
       </c>
@@ -1021,7 +1030,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="12">
         <v>2</v>
       </c>
@@ -1032,7 +1041,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="12">
         <v>3</v>
       </c>
@@ -1043,7 +1052,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="12">
         <v>4</v>
       </c>
@@ -1310,5 +1319,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>